<commit_message>
added a columns to the statistics tables for a mann whitney u test between in/out-paralogs
</commit_message>
<xml_diff>
--- a/data/humanParalogStatistics.xlsx
+++ b/data/humanParalogStatistics.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,21 @@
           <t>Corr PValue</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PValue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -471,6 +486,19 @@
         <v>-0.2726166334458298</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>out-paralog</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>in-paralog</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -507,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,6 +569,21 @@
           <t>Corr PValue</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PValue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -561,6 +604,19 @@
         <v>0.1788149768482298</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>out-paralog</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>in-paralog</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -597,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,6 +687,21 @@
           <t>Corr PValue</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PValue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -652,6 +723,19 @@
       </c>
       <c r="F2" t="n">
         <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>out-paralog</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>in-paralog</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>2.668072276074452e-42</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,6 +805,21 @@
           <t>Corr PValue</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PValue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -741,6 +840,19 @@
         <v>0.1088690243139833</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>out-paralog</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>in-paralog</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -777,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,6 +923,21 @@
           <t>Corr PValue</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PValue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -832,6 +959,19 @@
       </c>
       <c r="F2" t="n">
         <v>3.217500500113479e-18</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>out-paralog</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>in-paralog</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>8.655730744541496e-08</v>
       </c>
     </row>
     <row r="3">

</xml_diff>